<commit_message>
:up: cards criados - mat fin
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G374"/>
+  <dimension ref="A1:G387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6382,8 +6382,10 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="n">
-        <v>233</v>
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -6402,13 +6404,44 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ul&gt;
-	&lt;li&gt;ÍNDICES DE LIQUIDEZ &lt;ul&gt; &lt;li&gt;Índice de liquidez corrente = Ativo circulante/Passivo circulante&lt;/li&gt; &lt;li&gt;Indice de liquidez seca = (Ativo circulante – Estoques)/Passivo circulante&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;ÍNDICES DE ATIVIDADE &lt;ul&gt; &lt;li&gt;Giro do estoque = Custo das mercadorias vendidas/Estoque&lt;/li&gt; &lt;li&gt;Prazo médio de recebimento = Contas a receber de clientes/Valor diário médio das vendas&lt;/li&gt; &lt;li&gt;Prazo médio de recebimento = (Contas a receber de clientes x 360)/Vendas anuais&lt;/li&gt; &lt;li&gt;Prazo médio de pagamento = Fornecedores/Valor diário médio das compras&lt;/li&gt; &lt;li&gt;Prazo médio de pagamento = (Fornecedore x 360)/Compras anuais&lt;/li&gt; &lt;li&gt;Giro do ativo total = Vendas/Ativo total&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;ÍNDICES DE ENDIVIDAMENTO &lt;ul&gt; &lt;li&gt;Índice de endividamento geral = Passivo total/Ativo total&lt;/li&gt; &lt;li&gt;Índice de cobertura de juros = Lucro antes de juros e imposto de renda/Juros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;ÍNDICES DE RENTABILIDADE &lt;ul&gt; &lt;li&gt;Margem de lucro bruto = (Receita de vendas – Custo das mercadorias vendidas)/Receita de vendas = Lucro bruto/Receita de vendas&lt;/li&gt; &lt;li&gt;Margem de lucro operacional = Lucro operacional/Receita de vendas&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-&lt;/ul&gt;
-</t>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;ÍNDICES DE LIQUIDEZ&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Índice de liquidez corrente = $\frac{Ativo\ circulante}{Passivo\ circulante}$&lt;/li&gt;
+            &lt;li&gt;Índice de liquidez seca = $\frac{Ativo\ circulante\ –\ Estoques}{Passivo\ circulante}$&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;ÍNDICES DE ATIVIDADE&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Giro do estoque = $\frac{Custo\ das\ mercadorias\ vendidas}{Estoque}$&lt;/li&gt;
+            &lt;li&gt;Prazo médio de recebimento = $\frac{Contas\ a\ receber\ de\ clientes}{Valor\ diário\ médio\ das\ vendas}$&lt;/li&gt;
+            &lt;li&gt;Prazo médio de pagamento = $\frac{Fornecedores}{Valor\ diário\ médio\ das\ compras}$&lt;/li&gt;
+            &lt;li&gt;Giro do ativo total = $\frac{Vendas}{Ativo\ total}$&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;ÍNDICES DE ENDIVIDAMENTO&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Índice de endividamento geral = $\frac{Passivo\ total}{Ativo\ total}$&lt;/li&gt;
+            &lt;li&gt;Índice de cobertura de juros = $\frac{Lucro\ antes\ de\ juros\ e\ imposto\ de\ renda}{Juros}$&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;ÍNDICES DE RENTABILIDADE E RETORNO&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Margem de lucro bruto = $\frac{Lucro\ bruto}{Receita\ de\ vendas}$&lt;/li&gt;
+            &lt;li&gt;Margem de lucro operacional = $\frac{Lucro\ operacional}{Receita\ de\ vendas}$&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;ROE (&lt;i&gt;Return on Equity&lt;/i&gt; / Retorno do Patrimônio Líquido)&lt;/strong&gt; = $\frac{Lucro\ L\acute{\imath}quido}{Patrim\hat{o}nio\ L\acute{\imath}quido}$
+                &lt;ul&gt;
+                    &lt;li&gt;indica o resultado alcançado com os investimentos realizados pelos acionistas ordinários&lt;/li&gt;
+                &lt;/ul&gt;
+            &lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;ROA (&lt;i&gt;Return on Assets&lt;/i&gt; / Retorno sobre o Ativo)&lt;/strong&gt; = $\frac{Lucro\ L\acute{\imath}quido}{Ativo\ Total}$
+                &lt;ul&gt;
+                    &lt;li&gt;indica a eficiência global no uso dos ativos pela gestão da empresa&lt;/li&gt;
+                &lt;/ul&gt;
+            &lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -14881,8 +14914,10 @@
       </c>
     </row>
     <row r="259">
-      <c r="A259" t="n">
-        <v>352</v>
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -14902,7 +14937,7 @@
       <c r="E259" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;&lt;strong&gt;Conceito CAPM (Capital Asset Pricing Model)&lt;/strong&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito CAPM&lt;/strong&gt;
     &lt;ul&gt;
       &lt;li&gt;Modelo que determina o retorno esperado de um investimento com base no risco sistêmico.&lt;/li&gt;
       &lt;li&gt;Fórmula: $E[R] = R_f + \beta \cdot (R_m - R_f)$.&lt;/li&gt;
@@ -14911,19 +14946,24 @@
   &lt;li&gt;&lt;strong&gt;Cálculo para Carteiras (Portfólio)&lt;/strong&gt;
     &lt;ul&gt;
       &lt;li&gt;O Beta da carteira é a média ponderada dos Betas individuais.&lt;/li&gt;
-      &lt;li&gt;$\beta_{carteira} = (\% \text{Ativo A} \cdot \beta_A) + (\% \text{Ativo B} \cdot \beta_B)$.&lt;/li&gt;
+      &lt;li&gt;$\beta_{carteira} = (\%\ Ativo\ A \cdot \beta_A) + (\%\ Ativo\ B \cdot \beta_B)$.&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Premissas Importantes&lt;/strong&gt;
     &lt;ul&gt;
       &lt;li&gt;&lt;strong&gt;Taxa Livre de Risco ($R_f$):&lt;/strong&gt; Retorno de ativos sem risco de crédito.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Beta ($\beta$):&lt;/strong&gt; Se &gt; 1, o ativo é mais volátil que o mercado; se &lt; 1, é mais defensivo.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Prêmio de Risco:&lt;/strong&gt; A diferença $(R_m - R_f)$ representa a compensação por correr risco de mercado.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Beta ($\beta$):&lt;/strong&gt; Risco sistêmico comparado ao mercado (onde mercado = 1).
+        &lt;ul&gt;
+            &lt;li&gt;se $\beta &gt; 1$: ativo agressivo e mais volátil que o mercado (ex: se o risco for 30% superior ao do mercado, $\beta = 1,3$).&lt;/li&gt;
+            &lt;li&gt;se $\beta &lt; 1$: ativo defensivo e menos volátil que o mercado.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Prêmio de Risco:&lt;/strong&gt; A diferença $(R_m - R_f)$ representa a compensação global por correr risco de mercado.&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Dica para Concursos:&lt;/strong&gt;
     &lt;ul&gt;
-      &lt;li&gt;Cuidado para não confundir "Retorno de Mercado" ($R_m$) com "Prêmio de Risco" ($R_m - R_f$). A questão já deu a diferença (o prêmio) de 10%, facilitando o cálculo.&lt;/li&gt;
+      &lt;li&gt;Cuidado para não confundir "Retorno de Mercado" ($R_m$) com "Prêmio de Risco" ($R_m - R_f$). Se o enunciado fornece o "prêmio pelo risco", você deve multiplicar o Beta diretamente por esse valor, sem subtrair o $R_f$ dentro do parênteses.&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
 &lt;/ul&gt;</t>
@@ -21398,6 +21438,651 @@
         <v>0</v>
       </c>
     </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>469</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Curva de Phillips (Curto e Longo Prazo)</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Conceito Central&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;relaciona as taxas de inflação e desemprego em uma economia&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Curto Prazo&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;curva negativamente inclinada (presença de &lt;i&gt;trade-off&lt;/i&gt;)&lt;/li&gt;
+            &lt;li&gt;maior inflação resulta em menor desemprego (e vice-versa)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Longo Prazo&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;não há &lt;i&gt;trade-off&lt;/i&gt; (escolha) entre inflação e desemprego&lt;/li&gt;
+            &lt;li&gt;curva é uma reta &lt;strong&gt;vertical&lt;/strong&gt;&lt;/li&gt;
+            &lt;li&gt;posicionada na &lt;b&gt;Taxa Natural de Desemprego (NAIRU - &lt;i&gt;Non-Accelerating Inflation Rate of Unemployment&lt;/i&gt; / Taxa de Desemprego Não Aceleradora da Inflação)&lt;/b&gt;&lt;/li&gt;
+            &lt;li&gt;a inflação não afeta o nível de emprego estrutural&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>470</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Elasticidade-Preço da Demanda (EPD)</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Definição&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;mede a sensibilidade da quantidade demandada de um bem frente a variações no seu preço&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Fórmula Base&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;$EPD = |\frac{\%\ Varia\c{c}\tilde{a}o\ na\ Quantidade}{\%\ Varia\c{c}\tilde{a}o\ no\ Pre\c{c}o}|$&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Classificação do Resultado (Sempre em Módulo)&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;strong&gt;Elástica ($EPD &gt; 1$):&lt;/strong&gt; quantidade varia em proporção &lt;b&gt;maior&lt;/b&gt; que o preço (comum em bens supérfluos)&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;Inelástica ($EPD &lt; 1$):&lt;/strong&gt; quantidade varia em proporção &lt;b&gt;menor&lt;/b&gt; que o preço (comum em bens essenciais)&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;Unitária ($EPD = 1$):&lt;/strong&gt; variações proporcionais exatas&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Lógica de Cálculo&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;se o preço de um serviço aumenta 25% e a demanda cai 10%, o módulo da divisão é $|-10\% / +25\%| = |-0,4| = 0,4$. A demanda é inelástica.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>0</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>471</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Índices de Inflação: IPC vs. Deflator do PIB</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Índice de Preços ao Consumidor (IPC)&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;mede o custo de uma cesta &lt;b&gt;fixa&lt;/b&gt; de bens e serviços&lt;/li&gt;
+            &lt;li&gt;foco: produtos comprados por consumidores representativos (famílias)&lt;/li&gt;
+            &lt;li&gt;inclui &lt;b&gt;bens importados&lt;/b&gt; (desde que consumidos pelas famílias e presentes na cesta)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Deflator do PIB (Produto Interno Bruto)&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;mede o custo de todos os bens e serviços finais produzidos internamente no país&lt;/li&gt;
+            &lt;li&gt;cesta &lt;b&gt;variável&lt;/b&gt; (muda anualmente conforme a produção da economia)&lt;/li&gt;
+            &lt;li&gt;&lt;b&gt;não&lt;/b&gt; considera bens importados (pois não fazem parte da produção nacional)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>0</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>472</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Economias e Deseconomias de Escala</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Economia de Escala&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;ocorre no &lt;b&gt;longo prazo&lt;/b&gt;&lt;/li&gt;
+            &lt;li&gt;o Custo Total Médio (CTMe) &lt;b&gt;cai&lt;/b&gt; à medida que a quantidade produzida aumenta&lt;/li&gt;
+            &lt;li&gt;resultado da diluição dos custos fixos em um volume maior de produção&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Deseconomia de Escala&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;o Custo Total Médio (CTMe) &lt;b&gt;sobe&lt;/b&gt; com o aumento extremo da produção&lt;/li&gt;
+            &lt;li&gt;causada por ineficiências gerenciais, gargalos logísticos ou burocracia excessiva devido ao tamanho da operação&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Retornos Constantes de Escala&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;o Custo Total Médio (CTMe) se mantém &lt;b&gt;constante&lt;/b&gt; com a variação da produção&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>0</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>473</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Alavancagem Operacional e Financeira</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Alavancagem Operacional&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;relação direta com o aumento da estrutura de &lt;b&gt;Custos Fixos&lt;/b&gt; (ex: investir em expansão de capacidade produtiva fixa)&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;Impactos e Riscos:&lt;/strong&gt;
+                &lt;ul&gt;
+                    &lt;li&gt;aumenta o Ponto de Equilíbrio&lt;/li&gt;
+                    &lt;li&gt;eleva o &lt;b&gt;Risco Operacional&lt;/b&gt; da empresa&lt;/li&gt;
+                    &lt;li&gt;pequenas variações no volume de vendas passam a causar variações proporcionalmente maiores no lucro&lt;/li&gt;
+                &lt;/ul&gt;
+            &lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Alavancagem Financeira&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;relação com o uso de &lt;b&gt;Capital de Terceiros&lt;/b&gt; (dívidas) na estrutura de financiamento&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;Impactos e Riscos:&lt;/strong&gt;
+                &lt;ul&gt;
+                    &lt;li&gt;busca aumentar o retorno para o capital dos acionistas&lt;/li&gt;
+                    &lt;li&gt;aumenta o &lt;b&gt;Risco Financeiro&lt;/b&gt; devido à obrigatoriedade do pagamento de juros fixos&lt;/li&gt;
+                &lt;/ul&gt;
+            &lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>0</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>474</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Operações de Desconto: Teoria e Relações Conceituais</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceitos Iniciais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Nominal ($N$):&lt;/strong&gt; valor de face ou valor futuro do título[cite: 4].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Atual ($A$):&lt;/strong&gt; valor recebido antecipadamente, também designado Valor Descontado ou Valor Presente[cite: 4].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Desconto ($D$):&lt;/strong&gt; diferença absoluta entre o Valor Nominal e o Valor Atual ($D=N-A$)[cite: 4].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Racional (Por Dentro)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;a taxa de desconto incide sobre o &lt;strong&gt;Valor Atual&lt;/strong&gt; do título[cite: 6].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Comercial / Bancário (Por Fora)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;a taxa de desconto incide sobre o &lt;strong&gt;Valor Nominal&lt;/strong&gt; do título[cite: 6].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Relação Conceitual (Mesmo título, taxa e prazo)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;o Desconto Comercial será sempre &lt;strong&gt;maior&lt;/strong&gt; que o Desconto Racional ($D_{CS}&gt;D_{RS}$)[cite: 22, 26].&lt;/li&gt;
+      &lt;li&gt;o Valor Atual no Desconto Comercial será sempre &lt;strong&gt;menor&lt;/strong&gt; que o Valor Atual no Desconto Racional ($A_{CS}&lt;A_{RS}$)[cite: 22, 26].&lt;/li&gt;
+      &lt;li&gt;o Desconto Racional revela-se mais vantajoso para o proprietário do título, dado que proporciona um Valor Atual superior[cite: 24].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>0</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>475</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Fórmulas de Desconto Simples</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Racional Simples (Por Dentro)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Fórmula do Desconto:&lt;/strong&gt; $D_{RS}=A \times i \times t$[cite: 6, 25].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Atual:&lt;/strong&gt; $A=\frac{N}{(1+i \times t)}$[cite: 6, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Comercial Simples (Por Fora)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Fórmula do Desconto:&lt;/strong&gt; $D_{CS}=N \times i \times t$[cite: 7, 25].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Atual:&lt;/strong&gt; $A=N \times (1-i \times t)$[cite: 7, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Relação Matemática entre os Descontos Simples&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;conhecendo um dos descontos, pode obter-se o outro através da expressão: $D_{CS}=D_{RS} \times (1+i \times t)$[cite: 11, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>476</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Fórmulas de Desconto Composto</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Racional Composto (Por Dentro)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Atual:&lt;/strong&gt; $A=\frac{N}{(1+i)^t}$[cite: 14, 25].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cálculo do Desconto:&lt;/strong&gt; $D_{RC}=N-A$[cite: 14, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Desconto Comercial Composto (Por Fora)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Valor Atual:&lt;/strong&gt; $A=N \times (1-i)^t$[cite: 14, 25].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cálculo do Desconto:&lt;/strong&gt; $D_{CC}=N-A$[cite: 14, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>0</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais e Deslocamento no Tempo</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito Base&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;dois ou mais capitais com datas de resgate distintas são equivalentes se, ao serem transportados para uma mesma data focal à mesma taxa de juros, originarem valores idênticos[cite: 64, 87].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Regras de Deslocamento Temporal&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Deslocar para o futuro (Direita / Capitalização):&lt;/strong&gt; multiplica-se a parcela por $(1+i)^t$ em juros compostos, ou por $(1+i \times t)$ em juros simples[cite: 63, 87].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Deslocar para o passado (Esquerda / Descapitalização):&lt;/strong&gt; divide-se a parcela por $(1+i)^t$ em juros compostos, ou por $(1+i \times t)$ em juros simples[cite: 63, 87].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Propriedade Fundamental (Juros Compostos)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;em regime de Juros Compostos, a comparação e a equivalência de capitais &lt;strong&gt;não dependem&lt;/strong&gt; da data focal escolhida[cite: 64, 88]. Qualquer data na linha temporal validará a equivalência[cite: 64].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>0</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>479</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Taxa Efetiva em Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito de Taxa Efetiva&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;é a taxa de juros que, ao ser aplicada sobre o Valor Atual, gera o Valor Nominal no período considerado[cite: 18, 23].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Característica do Desconto Comercial&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;a taxa de desconto comercial &lt;strong&gt;não é&lt;/strong&gt; uma taxa efetiva, dado que incide sobre o Valor Nominal[cite: 19, 24].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fórmula de Conversão (Desconto Comercial Simples)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;$i_{ef}=\frac{i_{cs}}{1-i_{cs} \times t}$[cite: 18, 25].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>0</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>480</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Rendas Uniformes (Séries de Pagamento): Valor Atual (VA)</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito de Rendas Uniformes (Certas)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;sequência de fluxos de caixa em intervalos de tempo iguais, com parcelas constantes[cite: 70, 88].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Valor Atual de Rendas Postecipadas (Fim do período)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;$VA=P \times \left[ \frac{(1+i)^n-1}{i \times (1+i)^n} \right]$ ou $VA=P \times \left[ \frac{1-(1+i)^{-n}}{i} \right]$[cite: 71, 88].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Fator de Valor Atual:&lt;/strong&gt; $a_{n-i}=\left[ \frac{(1+i)^n-1}{i \times (1+i)^n} \right]$[cite: 73, 88]. O Fator de Recuperação de Capital (FRC) é o seu inverso: $FRC=\frac{1}{a_{n-i}}$[cite: 73, 88].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Valor Atual de Rendas Antecipadas (Início do período)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;a fórmula é idêntica à das rendas postecipadas, sendo no final multiplicada pelo fator de capitalização $(1+i)$[cite: 77, 88].&lt;/li&gt;
+      &lt;li&gt;$VA=P \times \left[ \frac{(1+i)^n-1}{i \times (1+i)^n} \right] \times (1+i)$[cite: 77].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>0</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>481</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Rendas Uniformes (Séries de Pagamento): Valor Futuro (VF)</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Valor Futuro de Rendas Postecipadas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;$VF=P \times \left[ \frac{(1+i)^n-1}{i} \right]$[cite: 74, 88].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Fator de Valor Futuro (Acumulação):&lt;/strong&gt; $S_{n-i}=\left[ \frac{(1+i)^n-1}{i} \right]$[cite: 76, 89]. O Fator de Formação de Capital (FFC) é o seu inverso: $FFC=\frac{1}{S_{n-i}}$[cite: 76, 89].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Valor Futuro de Rendas Antecipadas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;a expressão matemática do Valor Futuro para uma série antecipada é &lt;strong&gt;igual&lt;/strong&gt; à da série postecipada[cite: 78].&lt;/li&gt;
+      &lt;li&gt;a multiplicação adicional pelo fator $(1+i)$ verifica-se apenas no cálculo do Valor Atual[cite: 78].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>0</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>482</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Rendas Perpétuas (Termos Ilimitados)</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;fluxos de duração infinita, ou seja, sem um número de prestações passível de determinação exata[cite: 83, 89]. Na ausência de especificação no problema, assume-se a modalidade postecipada[cite: 84].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fórmulas do Valor Atual (VA)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Postecipadas:&lt;/strong&gt; $VA=\frac{P}{i}$[cite: 83, 89].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Postecipadas com crescimento ($g$):&lt;/strong&gt; $VA=\frac{P}{i-g}$[cite: 83, 89].&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Antecipadas:&lt;/strong&gt; $VA=\frac{P}{i} \times (1+i)$[cite: 84, 89].&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>0</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: resquicios de funcoes antigas apagados
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G410"/>
+  <dimension ref="A1:G412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23532,6 +23532,109 @@
         <v>0</v>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>508</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Distribuição Física (Outbound Logistics)</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Conceito Central&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;trata da movimentação, estocagem e processamento de pedidos dos &lt;b&gt;produtos finais&lt;/b&gt; (acabados) da firma&lt;/li&gt;
+            &lt;li&gt;foca no fluxo de saída: inicia na liberação da esteira de montagem fabril e vai até a entrega ao mercado/consumidor final&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Fronteiras e Escopo (Pegadinhas de Prova)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;não engloba o fluxo de entrada (recebimento de matérias-primas e insumos), que é função do Suprimento Físico (&lt;i&gt;Inbound Logistics&lt;/i&gt; / Administração de Materiais)&lt;/li&gt;
+            &lt;li&gt;não engloba a fabricação ou transformação da matéria-prima (Produção/Manufatura)&lt;/li&gt;
+            &lt;li&gt;é estruturada para &lt;b&gt;apoiar&lt;/b&gt; o Canal de Distribuição (este foca nas relações de vendas, marketing e troca de posse, sendo planejado primeiro)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Logística Empresarial Integrada&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;busca a unificação gerencial e de planejamento das frentes de abastecimento (&lt;i&gt;inbound&lt;/i&gt;) com a frente de distribuição física (&lt;i&gt;outbound&lt;/i&gt;)&lt;/li&gt;
+            &lt;li&gt;ambos os canais (suprimento e distribuição) apresentam grandes similaridades em suas atividades&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>0</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>509</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Logística de Suprimentos (Inbound Logistics / Administração de Materiais)</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Conceito Central&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;trata do fluxo de materiais, insumos e matérias-primas &lt;b&gt;dos fornecedores para a empresa&lt;/b&gt;&lt;/li&gt;
+            &lt;li&gt;foco no fluxo de entrada: vai da aquisição estruturada até a disponibilização do material para o início do processo de produção (manufatura)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Principais Atividades&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;seleção e negociação com fornecedores (compras / &lt;i&gt;procurement&lt;/i&gt;)&lt;/li&gt;
+            &lt;li&gt;transporte de suprimentos (da origem até a fábrica)&lt;/li&gt;
+            &lt;li&gt;recebimento e controle de qualidade de insumos&lt;/li&gt;
+            &lt;li&gt;armazenagem e gestão de estoques de matérias-primas&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Diferença Crucial (Inbound vs. Outbound)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;b&gt;Inbound:&lt;/b&gt; movimenta o que a empresa &lt;i&gt;precisa para produzir&lt;/i&gt; (foco na relação a montante / &lt;i&gt;upstream&lt;/i&gt; com fornecedores).&lt;/li&gt;
+            &lt;li&gt;&lt;b&gt;Outbound:&lt;/b&gt; movimenta o que a empresa &lt;i&gt;já produziu&lt;/i&gt; (foco na relação a jusante / &lt;i&gt;downstream&lt;/i&gt; com clientes).&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>0</v>
+      </c>
+      <c r="G412" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: flahscards de portugues reorganizados
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -18526,8 +18526,10 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" t="n">
-        <v>467</v>
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>467</t>
+        </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
@@ -18547,60 +18549,29 @@
       <c r="E318" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;&lt;b&gt;Conceito&lt;/b&gt;
-    &lt;ul&gt;
-      &lt;li&gt;Expressões que indicam parte de um todo
-        &lt;ul&gt;
-          &lt;li&gt;Ex: &lt;i&gt;a maioria de, a maior parte de, grande parte de, uma porção de, o resto de, metade de&lt;/i&gt;&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;Geralmente acompanhadas de um determinante (especificador)&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;b&gt;Regras de Concordância Verbal&lt;/b&gt;
-    &lt;ul&gt;
-      &lt;li&gt;&lt;b&gt;Determinante no Plural&lt;/b&gt; (Ex: &lt;i&gt;"dos alunos"&lt;/i&gt;)
-        &lt;ul&gt;
-          &lt;li&gt;A concordância é &lt;b&gt;facultativa&lt;/b&gt; (ambas as formas são corretas)&lt;/li&gt;
-          &lt;li&gt;&lt;b&gt;Concordância Gramatical (Rigorosa):&lt;/b&gt;
-            &lt;ul&gt;
-              &lt;li&gt;Verbo concorda com o &lt;b&gt;núcleo&lt;/b&gt; singular da expressão partitiva&lt;/li&gt;
-              &lt;li&gt;Ex: &lt;i&gt;A maioria dos candidatos &lt;u&gt;foi&lt;/u&gt; aprovada.&lt;/i&gt;&lt;/li&gt;
-            &lt;/ul&gt;
-          &lt;/li&gt;
-          &lt;li&gt;&lt;b&gt;Concordância Ideológica (Atrativa / Silepse de Número):&lt;/b&gt;
-            &lt;ul&gt;
-              &lt;li&gt;Verbo concorda com o &lt;b&gt;determinante&lt;/b&gt; no plural&lt;/li&gt;
-              &lt;li&gt;Ex: &lt;i&gt;A maioria dos candidatos &lt;u&gt;foram&lt;/u&gt; aprovados.&lt;/i&gt;&lt;/li&gt;
-            &lt;/ul&gt;
-          &lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;&lt;b&gt;Determinante no Singular ou Inexistente&lt;/b&gt; (Ex: &lt;i&gt;"do grupo"&lt;/i&gt;)
-        &lt;ul&gt;
-          &lt;li&gt;A concordância é &lt;b&gt;obrigatoriamente&lt;/b&gt; no singular&lt;/li&gt;
-          &lt;li&gt;Ex: &lt;i&gt;A maior parte da população &lt;u&gt;votou&lt;/u&gt;.&lt;/i&gt;&lt;/li&gt;
-          &lt;li&gt;Ex: &lt;i&gt;A maioria &lt;u&gt;decidiu&lt;/u&gt; ir embora.&lt;/i&gt;&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;b&gt;Expressões Correlatas (Mesma Lógica)&lt;/b&gt;
-    &lt;ul&gt;
-      &lt;li&gt;&lt;b&gt;Coletivos Partitivos&lt;/b&gt;
-        &lt;ul&gt;
-          &lt;li&gt;Ex: &lt;i&gt;um bando de, uma multidão de, um grupo de&lt;/i&gt;&lt;/li&gt;
-          &lt;li&gt;Seguem a mesma regra facultativa se o determinante for plural&lt;/li&gt;
-          &lt;li&gt;Ex: &lt;i&gt;Uma multidão de fãs &lt;u&gt;gritou / gritaram&lt;/u&gt;.&lt;/i&gt;&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;&lt;b&gt;Porcentagens e Frações&lt;/b&gt;
-        &lt;ul&gt;
-          &lt;li&gt;Verbo pode concordar com o &lt;b&gt;número&lt;/b&gt; ou com o &lt;b&gt;determinante&lt;/b&gt;&lt;/li&gt;
-          &lt;li&gt;Ex: &lt;i&gt;1% dos alunos &lt;u&gt;faltou / faltaram&lt;/u&gt;.&lt;/i&gt;&lt;/li&gt;
-          &lt;li&gt;Atenção: Se não houver determinante, concorda estritamente com o número (Ex: &lt;i&gt;1% &lt;u&gt;faltou&lt;/u&gt; / 2% &lt;u&gt;faltaram&lt;/u&gt;&lt;/i&gt;).&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;A Estrutura do Sujeito Partitivo&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O sujeito é formado por duas partes: o &lt;b&gt;Núcleo&lt;/b&gt; (ex: &lt;i&gt;A maioria&lt;/i&gt; - sempre singular) e o &lt;b&gt;Determinante&lt;/b&gt; (ex: &lt;i&gt;dos candidatos&lt;/i&gt; - que pode ser plural ou singular).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Regra 1: Determinante no Plural&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A concordância é &lt;b&gt;facultativa&lt;/b&gt;. Você tem dois caminhos igualmente corretos na prova:&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Caminho 1 (Concordar com o Núcleo):&lt;/b&gt; O verbo fica no singular. &lt;i&gt;Ex: A &lt;u&gt;maioria&lt;/u&gt; dos candidatos &lt;u&gt;foi&lt;/u&gt; aprovada.&lt;/i&gt;&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Caminho 2 (Concordar com o Determinante):&lt;/b&gt; O verbo fica no plural, atraído pela proximidade. &lt;i&gt;Ex: A maioria dos &lt;u&gt;candidatos foram&lt;/u&gt; aprovados.&lt;/i&gt;&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Regra 2: Determinante no Singular (ou Inexistente)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A concordância é &lt;b&gt;obrigatória no singular&lt;/b&gt;. Como não existe nenhuma palavra no plural para atrair o verbo, a regra facultativa deixa de existir.&lt;/li&gt;
+      &lt;li&gt;&lt;i&gt;Ex: A maior parte &lt;u&gt;da população votou&lt;/u&gt;.&lt;/i&gt;&lt;/li&gt;
+      &lt;li&gt;&lt;i&gt;Ex: A maioria &lt;u&gt;decidiu&lt;/u&gt; ir embora.&lt;/i&gt;&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Expressões Correlatas (Mesma Lógica)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Coletivos Partitivos:&lt;/b&gt; &lt;i&gt;um bando de, uma multidão de, um grupo de.&lt;/i&gt; Seguem a mesma regra facultativa se o determinante for plural. &lt;i&gt;Ex: Uma multidão de fãs &lt;u&gt;gritou / gritaram&lt;/u&gt;.&lt;/i&gt;&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Porcentagens e Frações:&lt;/b&gt; O verbo pode concordar com o número ou com o determinante. &lt;i&gt;Ex: 1% dos alunos &lt;u&gt;faltou / faltaram&lt;/u&gt;.&lt;/i&gt; (Se não houver determinante, concorda estritamente com o número: &lt;i&gt;1% &lt;u&gt;faltou&lt;/u&gt; / 2% &lt;u&gt;faltaram&lt;/u&gt;&lt;/i&gt;).&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
 &lt;/ul&gt;</t>

</xml_diff>

<commit_message>
:up: algumas cards criados - con esp - gest eco
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G361"/>
+  <dimension ref="A1:G370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21049,6 +21049,520 @@
         <v>0</v>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>511</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Gestão Económica e Modelo GECON</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Gestão económica&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;administração baseada em resultados económicos&lt;/li&gt;
+                &lt;li&gt;foco da avaliação de decisões
+                    &lt;ul&gt;
+                        &lt;li&gt;criação ou destruição de valor&lt;/li&gt;
+                        &lt;li&gt;comparação com a melhor alternativa disponível (custo de oportunidade)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Modelo GECON&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;lucro corretamente mensurado como medida de eficácia&lt;/li&gt;
+                &lt;li&gt;visão sistémica e integração&lt;/li&gt;
+                &lt;li&gt;pilares
+                    &lt;ul&gt;
+                        &lt;li&gt;modelo de gestão (crenças e valores)&lt;/li&gt;
+                        &lt;li&gt;processo de gestão (planeamento e controlo)&lt;/li&gt;
+                        &lt;li&gt;sistema de informação (mensuração pelo resultado económico)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>512</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Princípios da Engenharia Económica e EVA</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Engenharia económica&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;comparação monetária de alternativas de investimento e operação&lt;/li&gt;
+                &lt;li&gt;princípios de decisão
+                    &lt;ul&gt;
+                        &lt;li&gt;valor do dinheiro no tempo&lt;/li&gt;
+                        &lt;li&gt;incrementalidade (apenas fluxos que mudam com a decisão importam)&lt;/li&gt;
+                        &lt;li&gt;exclusão de custos afundados (gastos irrecuperáveis não influenciam opções futuras)&lt;/li&gt;
+                        &lt;li&gt;custo de oportunidade (retorno da alternativa preterida)&lt;/li&gt;
+                        &lt;li&gt;foco no fluxo de caixa efetivo&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;EVA (Valor Económico Agregado)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;criação de valor após remunerar o capital pelo custo de oportunidade&lt;/li&gt;
+                &lt;li&gt;fórmulas
+                    &lt;ul&gt;
+                        &lt;li&gt;EVA = Lucro operacional líquido de impostos - (Custo de capital × Capital investido)&lt;/li&gt;
+                        &lt;li&gt;EVA = Capital investido × (Retorno sobre o capital - Custo do capital)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>513</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Terminologia de Custos e Ciclo de Vida</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Classificação de custos&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;quanto ao volume
+                    &lt;ul&gt;
+                        &lt;li&gt;fixos (não mudam com a quantidade produzida na capacidade instalada)&lt;/li&gt;
+                        &lt;li&gt;variáveis (mudam proporcionalmente)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+                &lt;li&gt;quanto ao produto
+                    &lt;ul&gt;
+                        &lt;li&gt;diretos (mensuração objetiva)&lt;/li&gt;
+                        &lt;li&gt;indiretos (necessitam de rateio)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Ciclo de vida do projeto&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;implantação
+                    &lt;ul&gt;
+                        &lt;li&gt;Capex (despesas de capital e obras)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+                &lt;li&gt;operação
+                    &lt;ul&gt;
+                        &lt;li&gt;Opex (despesas recorrentes de funcionamento)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+                &lt;li&gt;desativação
+                    &lt;ul&gt;
+                        &lt;li&gt;custos de encerramento e descomissionamento&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>514</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Microeconomia e Ponto de Equilíbrio</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Elasticidade-preço da procura&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;sensibilidade da quantidade à variação de preço&lt;/li&gt;
+                &lt;li&gt;Ep = 0: perfeitamente inelástica&lt;/li&gt;
+                &lt;li&gt;0 &amp;lt; Ep &amp;lt; 1: inelástica&lt;/li&gt;
+                &lt;li&gt;Ep &amp;gt; 1: elástica&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Teoria da produção&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;lei dos rendimentos decrescentes (acréscimos marginais sucessivamente menores)&lt;/li&gt;
+                &lt;li&gt;ponto de encerramento (quando o preço cai abaixo do custo variável médio mínimo)&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Ponto de Equilíbrio (Nivelamento)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;Receita Total = Custo Total (lucro zero)&lt;/li&gt;
+                &lt;li&gt;quantidade = Custo Fixo / (Preço - Custo Variável Unitário)&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>0</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>515</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Estudo de Mercado e Procura</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Análise de mercado&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;bens finais (consumidor direto)&lt;/li&gt;
+                &lt;li&gt;bens intermediários (procura derivada da produção do bem final)&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Consumo Aparente (CA)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;CA = Produção Nacional + Importações - Exportações&lt;/li&gt;
+                &lt;li&gt;substitui a medição do consumo real por ignorar a variação de &lt;i&gt;stocks&lt;/i&gt;&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Projeção da procura futura&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;extrapolação de tendência histórica&lt;/li&gt;
+                &lt;li&gt;coeficientes de elasticidade
+                    &lt;ul&gt;
+                        &lt;li&gt;Mn = Mo × (1 + taxa populacional + Ey × taxa de rendimento - Ep × taxa de preço)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>516</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Engenharia de Projeto e Tecnologias</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Etapas da engenharia&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;ensaios preliminares e provas de conceito (mitigação de risco)&lt;/li&gt;
+                &lt;li&gt;seleção de processo e equipamentos&lt;/li&gt;
+                &lt;li&gt;construção civil e &lt;i&gt;layout&lt;/i&gt; espacial&lt;/li&gt;
+                &lt;li&gt;quantificação de insumos e mão de obra&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Seleção tecnológica&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;processo estruturado
+                    &lt;ul&gt;
+                        &lt;li&gt;definição de requisitos&lt;/li&gt;
+                        &lt;li&gt;prospeção tecnológica para avaliar maturidade&lt;/li&gt;
+                        &lt;li&gt;filtro de viabilidade local antes do contacto com fornecedores&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+                &lt;li&gt;distorções comuns
+                    &lt;ul&gt;
+                        &lt;li&gt;"seleção por lista telefónica" (escolha simplificada sem prospeção)&lt;/li&gt;
+                        &lt;li&gt;aquisição injustificada de bens importados intensivos em capital&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>517</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Investimentos e Financiamento</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Juros durante a construção&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;integram o investimento fixo (Capex) e não os custos operacionais&lt;/li&gt;
+                &lt;li&gt;cálculo com circularidade
+                    &lt;ul&gt;
+                        &lt;li&gt;I = Soma das parcelas / (1 - percentual financiado × taxa de juros)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Fontes de financiamento&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;internas
+                    &lt;ul&gt;
+                        &lt;li&gt;reinversão de lucros e provisões de depreciação&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+                &lt;li&gt;externas
+                    &lt;ul&gt;
+                        &lt;li&gt;capital próprio (sócios, investidores)&lt;/li&gt;
+                        &lt;li&gt;capital de terceiros (bancos, financiamentos)&lt;/li&gt;
+                    &lt;/ul&gt;
+                &lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>518</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Avaliação Financeira (VPL, TIR e VAUE)</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Taxa Mínima de Atratividade (TMA)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;custo de oportunidade do capital&lt;/li&gt;
+                &lt;li&gt;composição teórica: taxa livre de risco + prémio de risco + prémio de liquidez&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Valor Presente Líquido (VPL)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;soma dos fluxos de caixa descontados à TMA deduzida do investimento&lt;/li&gt;
+                &lt;li&gt;VPL &amp;gt; 0: aceitar projeto&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Taxa Interna de Retorno (TIR)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;taxa que anula o VPL&lt;/li&gt;
+                &lt;li&gt;TIR &amp;gt; TMA: aceitar projeto&lt;/li&gt;
+                &lt;li&gt;problema: múltiplas TIRs em fluxos com diversas inversões de sinal&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+        &lt;li&gt;&lt;b&gt;Valor Anual Uniforme Equivalente (VAUE)&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;transforma o VPL numa série de parcelas uniformes ao longo da vida útil&lt;/li&gt;
+                &lt;li&gt;indicado para a comparação de projetos com horizontes temporais diferentes&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>0</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>519</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Indicadores Agropecuários e Agroindustriais</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+        &lt;li&gt;&lt;b&gt;Medidas de ciclo produtivo&lt;/b&gt;
+            &lt;ul&gt;
+                &lt;li&gt;Renda Líquida (RL) = Receita Total - Custo Total&lt;/li&gt;
+                &lt;li&gt;Renda da Família (RF) = RL + Custo de Oportunidade + Custo do Trabalho Familiar&lt;/li&gt;
+                &lt;li&gt;Taxa de retorno do empreendedor = RL / Custo Total&lt;/li&gt;
+            &lt;/ul&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>0</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns cards criados - ind 4.0
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G370"/>
+  <dimension ref="A1:G381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21563,6 +21563,501 @@
         <v>0</v>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>520</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Internet das Coisas (IoT - Internet of Things)</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;rede de objetos físicos embarcados com sensores, &lt;i&gt;software&lt;/i&gt; e conectividade&lt;/li&gt;
+            &lt;li&gt;permite a comunicação e a troca de dados em tempo real entre máquinas e sistemas&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;monitoramento contínuo do chão de fábrica&lt;/li&gt;
+            &lt;li&gt;rastreabilidade completa de ativos e materiais&lt;/li&gt;
+            &lt;li&gt;base para a manutenção preditiva&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>0</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>521</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Sistemas Ciberfísicos (CPS - Cyber-Physical Systems)</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;integração de processos computacionais e físicos&lt;/li&gt;
+            &lt;li&gt;computadores e redes monitoram e controlam os processos físicos com &lt;i&gt;loops&lt;/i&gt; de &lt;i&gt;feedback&lt;/i&gt;&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;criação de fábricas inteligentes (&lt;i&gt;smart factories&lt;/i&gt;)&lt;/li&gt;
+            &lt;li&gt;descentralização da tomada de decisão&lt;/li&gt;
+            &lt;li&gt;adaptação autônoma das máquinas a mudanças nas condições de operação&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>0</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>522</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Computação em Nuvem (Cloud Computing)</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;fornecimento de serviços de computação via internet&lt;/li&gt;
+            &lt;li&gt;inclui servidores, armazenamento, bancos de dados, redes e &lt;i&gt;software&lt;/i&gt;&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;redução de custos com infraestrutura local de TI (Tecnologia da Informação)&lt;/li&gt;
+            &lt;li&gt;escalabilidade rápida de armazenamento e processamento&lt;/li&gt;
+            &lt;li&gt;acesso remoto e centralizado a dados de múltiplas plantas industriais&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>0</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>523</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Big Data e Analytics (Megadados e Análise de Dados)</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;coleta e análise de conjuntos de dados massivos e complexos&lt;/li&gt;
+            &lt;li&gt;extração de valor e padrões a partir do volume, velocidade e variedade de informações&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;otimização da qualidade da produção em tempo real&lt;/li&gt;
+            &lt;li&gt;identificação de gargalos operacionais invisíveis a análises tradicionais&lt;/li&gt;
+            &lt;li&gt;previsão de demanda com maior precisão e ajuste de capacidade produtiva&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>0</v>
+      </c>
+      <c r="G374" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>524</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Simulação e Gêmeos Digitais (Digital Twins)</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;réplica virtual exata de um produto, processo ou sistema físico&lt;/li&gt;
+            &lt;li&gt;alimentada com dados em tempo real via IoT&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;testes e otimizações de &lt;i&gt;layout&lt;/i&gt; e processos sem interrupção da linha física&lt;/li&gt;
+            &lt;li&gt;redução do tempo e custo de comissionamento de novos equipamentos&lt;/li&gt;
+            &lt;li&gt;simulação de cenários de falha para treinamento e mitigação de riscos&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>525</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Manufatura Aditiva (Impressão 3D)</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;criação de objetos tridimensionais a partir de modelos digitais&lt;/li&gt;
+            &lt;li&gt;adição sucessiva de camadas de material (plástico, metal, resina)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;prototipagem rápida e barateamento do desenvolvimento de produtos&lt;/li&gt;
+            &lt;li&gt;produção de lotes unitários ou peças de reposição sob demanda&lt;/li&gt;
+            &lt;li&gt;redução drástica de perdas e resíduos de matéria-prima comparada à usinagem tradicional&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>0</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>526</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Robótica Autônoma</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;robôs industriais com inteligência artificial para agir sem intervenção humana direta&lt;/li&gt;
+            &lt;li&gt;inclui robôs colaborativos (&lt;i&gt;cobots&lt;/i&gt;) que interagem de forma segura com operadores&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;assunção de tarefas repetitivas, insalubres ou de alta precisão&lt;/li&gt;
+            &lt;li&gt;aumento da flexibilidade da linha de montagem&lt;/li&gt;
+            &lt;li&gt;redução de acidentes de trabalho e de custos operacionais de longo prazo&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>0</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>527</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Segurança Cibernética (Cybersecurity)</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;proteção de sistemas, redes e programas contra ataques digitais&lt;/li&gt;
+            &lt;li&gt;garantia de integridade, confidencialidade e disponibilidade dos dados&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;proteção de dados industriais sensíveis e propriedade intelectual&lt;/li&gt;
+            &lt;li&gt;prevenção contra paralisações de fábrica causadas por &lt;i&gt;ransomware&lt;/i&gt; (&lt;i&gt;software&lt;/i&gt; de extorsão)&lt;/li&gt;
+            &lt;li&gt;garantia de operação contínua e segura dos sistemas ciberfísicos e maquinários&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>0</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>528</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Integração de Sistemas (Horizontal e Vertical)</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Horizontal: integração de dados entre fornecedores, empresa e clientes ao longo da cadeia de valor&lt;/li&gt;
+            &lt;li&gt;Vertical: integração de dados entre os diferentes níveis hierárquicos da empresa (do chão de fábrica ao ERP corporativo - &lt;i&gt;Enterprise Resource Planning&lt;/i&gt; / Planejamento de Recursos Empresariais)&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;fluxo de informações contínuo e sem silos departamentais&lt;/li&gt;
+            &lt;li&gt;agilidade na resposta a atrasos de fornecimento ou picos de demanda&lt;/li&gt;
+            &lt;li&gt;alinhamento total entre a execução física e o planejamento estratégico&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>0</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>529</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Inteligência Artificial (IA - Artificial Intelligence)</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;simulação de capacidades cognitivas humanas por sistemas computacionais&lt;/li&gt;
+            &lt;li&gt;engloba raciocínio, resolução de problemas, perceção e tomada de decisão&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;orquestração inteligente e autónoma de toda a cadeia de suprimentos&lt;/li&gt;
+            &lt;li&gt;sistemas de visão computacional avançada para inspeção de qualidade&lt;/li&gt;
+            &lt;li&gt;otimização instantânea de rotas, consumo energético e alocação de recursos&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>0</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>530</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Machine Learning (ML) / Aprendizado de Máquina</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;subcampo da IA focado em algoritmos que aprendem empiricamente com os dados&lt;/li&gt;
+            &lt;li&gt;permite que os sistemas melhorem o seu desempenho sem programação explícita para cada nova situação&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Impacto na produção&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;coração da manutenção preditiva, cruzando dados históricos para prever falhas antes que ocorram&lt;/li&gt;
+            &lt;li&gt;identificação de padrões ocultos e anomalias em grandes volumes de informação gerados pelo &lt;i&gt;Big Data&lt;/i&gt;&lt;/li&gt;
+            &lt;li&gt;ajuste autónomo e contínuo de parâmetros de maquinário para maximizar o rendimento e minimizar perdas&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns cards criados - all
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G393"/>
+  <dimension ref="A1:G399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13857,8 +13857,10 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" t="n">
-        <v>354</v>
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -13878,23 +13880,25 @@
       <c r="E231" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;&lt;strong&gt;Conceitos de Verbo para o Cebraspe&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;&lt;strong&gt;Pretérito Perfeito do Subjuntivo (Tenha Prevalecido):&lt;/strong&gt; Expressa um fato passado concluído em relação a um momento presente.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Presente do Indicativo (É):&lt;/strong&gt; Utilizado aqui para expressar uma definição conceitual e permanente (Presente Atemporal).&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Desconstruindo a Pegadinha&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;&lt;strong&gt;Presente Histórico:&lt;/strong&gt; &lt;u&gt;Não ocorre&lt;/u&gt; neste texto. Ele serve para "trazer o passado para o presente" em narrações, o que não é o caso de um manual técnico.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Paralelismo Temporal:&lt;/strong&gt; Não exige que todos os verbos estejam no mesmo tempo, mas sim que a relação entre eles seja lógica. No texto, a relação é: "Embora algo tenha ocorrido (passado), o fato é (presente)...".&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Dica de Ouro:&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;Sempre que a banca afirmar que um verbo é "Presente Histórico", verifique se o texto está contando uma história antiga. Se for um texto dissertativo/informativo como este, quase nunca será presente histórico.&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;1. Presente Pontual ou Habitual&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Indica uma ação que ocorre no momento da fala ou uma rotina/hábito contínuo.&lt;/li&gt;
+            &lt;li&gt;&lt;i&gt;Exemplo:&lt;/i&gt; "Eu &lt;b&gt;estudo&lt;/b&gt; todos os dias para o concurso."&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;2. Presente Atemporal (Verdade Universal / Validade Permanente)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Indica fatos incontestáveis, leis científicas, provérbios ou afirmações filosóficas. &lt;b&gt;Atribui validade permanente à afirmação.&lt;/b&gt;&lt;/li&gt;
+            &lt;li&gt;&lt;i&gt;Exemplos:&lt;/i&gt; "A água &lt;b&gt;ferve&lt;/b&gt; a 100 graus." / "O tempo é um imperador que &lt;b&gt;diz&lt;/b&gt; que &lt;b&gt;passa&lt;/b&gt;, quando quem passa &lt;b&gt;somos&lt;/b&gt; nós."&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;3. Presente Histórico&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Utiliza o tempo presente para narrar, com maior vivacidade e proximidade, fatos que já aconteceram e foram concluídos no passado.&lt;/li&gt;
+            &lt;li&gt;&lt;i&gt;Exemplo:&lt;/i&gt; "Em 1500, Cabral &lt;b&gt;chega&lt;/b&gt; ao Brasil e &lt;b&gt;descobre&lt;/b&gt; novas terras."&lt;/li&gt;
+            &lt;li&gt;&lt;b&gt;Dica de Ouro:&lt;/b&gt; Se for um texto técnico, dissertativo ou legal, dificilmente será presente histórico. Este recurso é típico de narrativas e crónicas.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -22720,6 +22724,257 @@
         <v>0</v>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>544</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Lei 13.303 - 2016</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Dispensa de Licitação: Contratação de Remanescente</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;É &lt;b&gt;dispensável&lt;/b&gt; a licitação para contratação de remanescente de obra, serviço ou fornecimento decorrente de rescisão contratual ou distrato.&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Requisitos obrigatórios para o novo contratado:&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Respeitar a &lt;b&gt;ordem de classificação&lt;/b&gt; da licitação anterior.&lt;/li&gt;
+            &lt;li&gt;Aceitar as &lt;b&gt;mesmas condições&lt;/b&gt; do contrato encerrado.&lt;/li&gt;
+            &lt;li&gt;Manter obrigatoriamente o &lt;b&gt;preço&lt;/b&gt;, devidamente corrigido.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>0</v>
+      </c>
+      <c r="G394" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>545</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Regressão Linear Múltipla</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Regressão Linear Múltipla: Equação, Pressupostos e Multicolinearidade</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Equação:&lt;/b&gt; $Y = \alpha + \beta_1 x_1 + \beta_2 x_2 + ... + \beta_k x_k + \epsilon$. Baseia-se no princípio &lt;i&gt;ceteris paribus&lt;/i&gt;, em que se estima o efeito de uma variável independente mantendo os outros fatores fixos.&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Pressupostos dos Erros ($\epsilon$):&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Média nula: $E(\epsilon_i) = 0$.&lt;/li&gt;
+            &lt;li&gt;Homocedasticidade: a variância do erro deve ser constante, independentemente do valor de $X$ ($Var(\epsilon_i) = \sigma^2$).&lt;/li&gt;
+            &lt;li&gt;Ausência de autocorrelação: os erros cometidos pelo modelo são independentes e não se correlacionam ($corr(\epsilon_i, \epsilon_j) = 0$).&lt;/li&gt;
+            &lt;li&gt;Normalidade: os erros têm distribuição normal.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Multicolinearidade:&lt;/b&gt; Ocorre quando há relação linear (alta correlação) entre as variáveis independentes, o que pode tornar a estimativa dos parâmetros insignificante.&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Graus de Liberdade (GL):&lt;/b&gt; Para $p$ parâmetros estimados (incluindo o intercepto), o GL do Modelo é $p-1$, o GL dos Resíduos é $n-p$ e o GL Total é $n-1$.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>0</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>546</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Regressão Linear Múltipla</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Variáveis Binárias (Dummies)</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Conceito:&lt;/b&gt; Assumem valores $0$ ou $1$ e são utilizadas para indicar a presença ou ausência de uma característica, incorporando aspetos qualitativos ao modelo (ex: sexo, estações do ano).&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Regra das Categorias:&lt;/b&gt; Para representar uma variável qualitativa com $n$ categorias, é necessário utilizar $n - 1$ variáveis binárias (a exclusão de uma categoria serve de referência para evitar ponderações arbitrárias).&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Aplicação:&lt;/b&gt; Quando incluídas diretamente no modelo, objetivam estimar diferenças no intercepto. Se usadas interagindo com outras variáveis explicativas, objetivam indicar diferenças na inclinação da reta de regressão para diferentes grupos.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>547</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Regressão Linear Múltipla</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Problema da Especificação e Teste RESET (Ramsey)</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Problema de Especificação:&lt;/b&gt; Erro na escolha do modelo matemático (linear, exponencial, polinomial) ou falha na determinação de quais variáveis independentes devem ser incluídas.
+        &lt;ul&gt;
+            &lt;li&gt;&lt;b&gt;Omissão de variável relevante:&lt;/b&gt; Torna as estimativas dos parâmetros tendenciosas (enviesadas).&lt;/li&gt;
+            &lt;li&gt;&lt;b&gt;Inclusão de variável desnecessária (irrelevante):&lt;/b&gt; As estimativas permanecem não-tendenciosas, mas a variância dos estimadores é aumentada.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Teste RESET (Ramsey):&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Adiciona polinómios quadráticos e cúbicos aos valores estimados pelo método dos mínimos quadrados (MQO) para detetar erros de especificação ou ausência de não linearidades importantes.&lt;/li&gt;
+            &lt;li&gt;Hipótese Nula ($H_0$): indica que o modelo original foi especificado corretamente. Rejeitar $H_0$ (quando $F_{calculado} &gt; F_{critico}$) significa que há erro de especificação.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>548</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Regressão Linear Múltipla</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Transformação de Box-Cox</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Objetivo:&lt;/b&gt; É uma transformação de potência aplicada para corrigir a não normalidade dos dados e estabilizar a variância, corrigindo a heterocedasticidade.&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Fórmula Base:&lt;/b&gt; $X^{(\lambda)} = \frac{X^\lambda - 1}{\lambda}$ ou simplificadamente $X^\lambda$ (para $\lambda \neq 0$).&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Caso Especial:&lt;/b&gt; Quando o parâmetro $\lambda = 0$, a transformação aplicada deve ser logarítmica ($X^{(0)} = \log(X)$).&lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Condição:&lt;/b&gt; A transformação de Box e Cox é definida apenas para variáveis com valores estritamente positivos ($X &gt; 0$).&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>0</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>549</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Reescritura: Invenção de Nexo, Modalização e Esvaziamento Semântico</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;b&gt;Invenção de Nexo (Relação Lógica Inexistente)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Transformar duas orações independentes (fatos que somam forças) em uma relação de subordinação (inserindo conectivos de causa/condição como &lt;i&gt;"considerando"&lt;/i&gt; ou &lt;i&gt;"já que"&lt;/i&gt;). Isso cria uma relação de dependência que o autor não escreveu.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Mudança de Modalização (Fato vs. Opinião)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Trocar uma afirmação categórica/objetiva (ex: &lt;i&gt;"é um sucesso"&lt;/i&gt;) por uma expressão de percepção ou consenso social (ex: &lt;i&gt;"já são aceitas como um sucesso"&lt;/i&gt;). Isso enfraquece a certeza da frase original.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;b&gt;Esvaziamento Semântico (Omissão de Palavras-Chave)&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Retirar adjetivos ou advérbios com peso argumentativo (ex: &lt;i&gt;"comprovado"&lt;/i&gt;, &lt;i&gt;"sempre"&lt;/i&gt;) atenua o argumento e constitui erro direto de sentido.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;hr&gt;
+    &lt;li&gt;&lt; ATENÇÃO: Particularidade CEBRASPE (Visão de "Coerência Global")&lt;/b&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Para o Cebraspe, cometer os erros acima não altera apenas o "sentido". Eles consideram que isso destrói a &lt;b&gt;macroestrutura argumentativa&lt;/b&gt; do autor e dão o item como ERRADO mesmo que o enunciado pergunte apenas se a &lt;i&gt;"coerência"&lt;/i&gt; foi mantida.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>0</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>